<commit_message>
Update menu: 93 item sesuai daftar menu resmi Madam Lily
Kategori: Bubur Ayam, Ayam Kalasan, Ayam Kuning, Nasi Spesial,
Soto Sop, Baso, Nasi Kuning, Nasi Uduk, Cemilan, Kerupuk,
Minuman, Rokok Cukai, Rokok Lokal.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/menu.xlsx
+++ b/data/menu.xlsx
@@ -439,9 +439,9 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
@@ -504,17 +504,21 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>BUBUR AYAM</t>
+          <t>BUBUR AYAM BIASA</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>10000</v>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BUBUR AYAM</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>🍚</t>
+          <t>🥡</t>
         </is>
       </c>
     </row>
@@ -534,7 +538,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>BUBUR AYAM TELUR</t>
+          <t>BUBUR AYAM JUMBO</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -544,7 +548,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>🍚</t>
+          <t>🥡</t>
         </is>
       </c>
     </row>
@@ -564,17 +568,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>BUBUR AYAM CEKER</t>
+          <t>TELUR ASIN</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>12000</v>
+        <v>2000</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>🍚</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -594,17 +598,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>BUBUR POLOS</t>
+          <t>SATE KULIT</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>7000</v>
+        <v>3000</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>🍚</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -624,17 +628,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BUBUR KACANG IJO</t>
+          <t>SATE USUS</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>7000</v>
+        <v>3000</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>🍚</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -649,22 +653,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AYAM KALASAN</t>
+          <t>BUBUR AYAM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AYAM KALASAN DADA</t>
+          <t>SATE ATI</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>20000</v>
+        <v>3000</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>🍗</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -679,22 +683,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AYAM KALASAN</t>
+          <t>BUBUR AYAM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AYAM KALASAN PAHA</t>
+          <t>SATE AMPLA</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>20000</v>
+        <v>3000</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>🍗</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -709,22 +713,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AYAM KALASAN</t>
+          <t>BUBUR AYAM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AYAM KALASAN SAYAP</t>
+          <t>SATE JANTUNG</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>15000</v>
+        <v>3000</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>🍗</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -739,22 +743,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AYAM KALASAN</t>
+          <t>BUBUR AYAM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NASI AYAM KALASAN DADA</t>
+          <t>TELUR PUYUH</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>25000</v>
+        <v>3000</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>🍗</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -774,13 +778,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NASI AYAM KALASAN PAHA</t>
+          <t>KALASAN DADA+NASI</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+        <v>12000</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>KALASAN DADA NASI</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
@@ -804,13 +812,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NASI AYAM KALASAN SAYAP</t>
+          <t>KALASAN PAHA+NASI</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+        <v>12000</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>KALASAN PAHA NASI</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
@@ -829,19 +841,23 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AYAM KUNING</t>
+          <t>AYAM KALASAN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>AYAM KUNING DADA</t>
+          <t>KALASAN DADA</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>18000</v>
+        <v>10000</v>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -859,19 +875,23 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AYAM KUNING</t>
+          <t>AYAM KALASAN</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>AYAM KUNING PAHA</t>
+          <t>KALASAN PAHA</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>18000</v>
+        <v>10000</v>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -894,13 +914,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AYAM KUNING SAYAP</t>
+          <t>KUNING DADA+NASI</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>13000</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+        <v>12000</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>KUNING DADA NASI</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
@@ -924,13 +948,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NASI AYAM KUNING DADA</t>
+          <t>KUNING PAHA+NASI</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>23000</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
+        <v>12000</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>KUNING PAHA NASI</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
@@ -954,14 +982,18 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NASI AYAM KUNING PAHA</t>
+          <t>KUNING DADA</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>23000</v>
+        <v>10000</v>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -984,14 +1016,18 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>NASI AYAM KUNING SAYAP</t>
+          <t>KUNING PAHA</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>18000</v>
+        <v>10000</v>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -1009,28 +1045,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>AYAM KUNING</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NASI GORENG</t>
+          <t>TEMPE KUNING</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>13000</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>NASGOR</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
+        <v>2000</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>tambahan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1043,28 +1075,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>AYAM KUNING</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>NASI GORENG TELUR</t>
+          <t>TAHU KUNING</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>NASGOR TELUR</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
+        <v>2000</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>tambahan</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1082,21 +1110,21 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NASI GORENG AYAM</t>
+          <t>AYAM PENYET CABE IJO</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>18000</v>
+        <v>16000</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>NASGOR AYAM</t>
+          <t>PENYET CABE IJO</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍗</t>
         </is>
       </c>
     </row>
@@ -1116,21 +1144,21 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NASI GORENG SPESIAL</t>
+          <t>NASI TELOR CHARSIU AYAM</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>20000</v>
+        <v>12000</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>NASGOR SPESIAL</t>
+          <t>NASI CHARSIU</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🌚</t>
         </is>
       </c>
     </row>
@@ -1150,21 +1178,21 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MIE GORENG</t>
+          <t>NASI AYAM SEREH</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>13000</v>
+        <v>12000</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>MIEGOR</t>
+          <t>AYAM SEREH</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍗</t>
         </is>
       </c>
     </row>
@@ -1179,26 +1207,26 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MIE GORENG TELUR</t>
+          <t>SOTO DAGING+NASI</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>15000</v>
+        <v>14000</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>MIEGOR TELUR</t>
+          <t>SOTO DAGING NASI</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1213,26 +1241,26 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MIE GORENG AYAM</t>
+          <t>SOTO TETELAN+NASI</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>18000</v>
+        <v>12000</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>MIEGOR AYAM</t>
+          <t>SOTO TETELAN NASI</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1247,26 +1275,26 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MIE GORENG SPESIAL</t>
+          <t>SOTO AYAM+NASI</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>20000</v>
+        <v>14000</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MIEGOR SPESIAL</t>
+          <t>SOTO AYAM NASI</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1281,26 +1309,26 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>KWETIAU GORENG</t>
+          <t>SOP DAGING+NASI</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>13000</v>
+        <v>14000</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>KWETIAW</t>
+          <t>SOP DAGING NASI</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1315,22 +1343,26 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>KWETIAU GORENG TELUR</t>
+          <t>SOP TETELAN+NASI</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
+        <v>12000</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SOP TETELAN NASI</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1345,22 +1377,26 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>KWETIAU GORENG AYAM</t>
+          <t>SOP AYAM+NASI</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
+        <v>14000</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>SOP AYAM NASI</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1375,22 +1411,26 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>KWETIAU GORENG SPESIAL</t>
+          <t>SOTO DAGING</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>20000</v>
+        <v>12000</v>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1405,22 +1445,26 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>BIHUN GORENG</t>
+          <t>SOTO TETELAN</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>13000</v>
+        <v>10000</v>
       </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1435,22 +1479,26 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>BIHUN GORENG TELUR</t>
+          <t>SOTO AYAM</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1465,22 +1513,26 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>BIHUN GORENG AYAM</t>
+          <t>SOP DAGING</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>18000</v>
+        <v>12000</v>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1495,22 +1547,26 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>BIHUN GORENG SPESIAL</t>
+          <t>SOP TETELAN</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1525,22 +1581,26 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>SOTO SOP</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>NASI CAMPUR</t>
+          <t>SOP AYAM</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>tanpa nasi</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍲</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1615,26 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>NASI SPESIAL</t>
+          <t>BASO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>NASI CAMPUR SPESIAL</t>
+          <t>BASO RACIK MIE+BIHUN</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
+        <v>14000</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>BASO RACIK MIE BIHUN,BAKSO RACIK</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍥</t>
         </is>
       </c>
     </row>
@@ -1585,22 +1649,26 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SOTO SOP</t>
+          <t>BASO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>SOTO AYAM</t>
+          <t>BASO RACIK NASI</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F37" t="inlineStr"/>
+        <v>14000</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>BAKSO RACIK NASI</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>🍲</t>
+          <t>🍥</t>
         </is>
       </c>
     </row>
@@ -1615,22 +1683,26 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SOTO SOP</t>
+          <t>NASI KUNING</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>SOTO DAGING</t>
+          <t>NASI KUNING</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
+        <v>7000</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>NASKU</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>🍲</t>
+          <t>🥚</t>
         </is>
       </c>
     </row>
@@ -1645,22 +1717,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SOTO SOP</t>
+          <t>NASI KUNING</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SOP AYAM</t>
+          <t>NASI KUNING JUMBO</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>🍲</t>
+          <t>🥚</t>
         </is>
       </c>
     </row>
@@ -1675,22 +1747,26 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SOTO SOP</t>
+          <t>NASI KUNING</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>SOP DAGING</t>
+          <t>NASI KUNING AYAM KALASAN</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
+        <v>15000</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>NASKU KALASAN</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>🍲</t>
+          <t>🥚</t>
         </is>
       </c>
     </row>
@@ -1705,22 +1781,26 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SOTO SOP</t>
+          <t>NASI KUNING</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>SOP IGA</t>
+          <t>NASI KUNING AYAM KUNING</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
+        <v>15000</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>NASKU KUNING</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>🍲</t>
+          <t>🥚</t>
         </is>
       </c>
     </row>
@@ -1735,22 +1815,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SOTO SOP</t>
+          <t>NASI UDUK</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>RAWON</t>
+          <t>NASI UDUK</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>20000</v>
+        <v>7000</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>🍲</t>
+          <t>🍚</t>
         </is>
       </c>
     </row>
@@ -1765,26 +1845,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>BASO</t>
+          <t>NASI UDUK</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>BASO KUAH</t>
+          <t>NASI UDUK JUMBO</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>13000</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>BAKSO</t>
-        </is>
-      </c>
+        <v>12000</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍚</t>
         </is>
       </c>
     </row>
@@ -1799,22 +1875,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>BASO</t>
+          <t>NASI UDUK</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>BASO GORENG</t>
+          <t>NASI UDUK AYAM KALASAN</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>13000</v>
+        <v>15000</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍚</t>
         </is>
       </c>
     </row>
@@ -1829,22 +1905,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BASO</t>
+          <t>NASI UDUK</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>BASO KUAH SPESIAL</t>
+          <t>NASI UDUK AYAM KUNING</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍚</t>
         </is>
       </c>
     </row>
@@ -1859,22 +1935,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>BASO</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>BASO TAHU</t>
+          <t>CAKWE</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>10000</v>
+        <v>1000</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -1889,22 +1965,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BASO</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>MIE AYAM</t>
+          <t>BAKWAN</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>13000</v>
+        <v>1000</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -1919,22 +1995,22 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BASO</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>MIE AYAM BASO</t>
+          <t>RISOL SAYUR</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>15000</v>
+        <v>3000</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>🍜</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -1949,26 +2025,22 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NASI KUNING</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>NASI KUNING</t>
+          <t>PASTEL</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>NASKU</t>
-        </is>
-      </c>
+        <v>3000</v>
+      </c>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -1983,22 +2055,22 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>NASI KUNING</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>NASI KUNING TELUR</t>
+          <t>LUMPIA BIHUN</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>12000</v>
+        <v>3000</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -2013,22 +2085,26 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>NASI KUNING</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>NASI KUNING AYAM</t>
+          <t>PISCOK</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F51" t="inlineStr"/>
+        <v>3000</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>PISANG COKLAT</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍫</t>
         </is>
       </c>
     </row>
@@ -2043,22 +2119,22 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>NASI KUNING</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>NASI KUNING SPESIAL</t>
+          <t>RISOL MAYO</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>18000</v>
+        <v>5000</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -2073,22 +2149,22 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>NASI UDUK</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>NASI UDUK</t>
+          <t>LEMPER</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -2103,22 +2179,22 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>NASI UDUK</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>NASI UDUK TELUR</t>
+          <t>LEMPER PEDES</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>12000</v>
+        <v>5000</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -2133,22 +2209,22 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>NASI UDUK</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>NASI UDUK AYAM</t>
+          <t>LOPIS</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -2163,22 +2239,22 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>NASI UDUK</t>
+          <t>CEMILAN</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>NASI UDUK SPESIAL</t>
+          <t>PUTU AYU</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>18000</v>
+        <v>5000</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>🍛</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2274,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>TAHU GORENG</t>
+          <t>ONGOL ONGOL</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -2228,7 +2304,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>TEMPE GORENG</t>
+          <t>LAPIS PEPE COKLAT</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2258,7 +2334,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>PISANG GORENG</t>
+          <t>LAPIS PEPE PANDAN</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -2268,7 +2344,7 @@
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>🍌</t>
+          <t>🍢</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2364,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>SINGKONG GORENG</t>
+          <t>DADAR GULUNG</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2318,11 +2394,11 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>RISOL</t>
+          <t>BUBUR KETAN HITAM</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
@@ -2348,13 +2424,17 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>PASTEL</t>
+          <t>BUBUR KACANG HIJAU</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F62" t="inlineStr"/>
+        <v>5000</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>BUBUR KACANG IJO</t>
+        </is>
+      </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
@@ -2378,7 +2458,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>LUMPIA</t>
+          <t>BUBUR SUM SUM</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -2408,17 +2488,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>MARTABAK TELUR</t>
+          <t>PUDING COKLAT</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>🥘</t>
+          <t>🍮</t>
         </is>
       </c>
     </row>
@@ -2433,22 +2513,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CEMILAN</t>
+          <t>KERUPUK</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GORENGAN CAMPUR</t>
+          <t>KERUPUK GENDAR</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>🍢</t>
+          <t>🍘</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2578,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>KERUPUK KULIT</t>
+          <t>KERUPUK PANGSIT</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -2528,13 +2608,17 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>KERUPUK MERAH</t>
+          <t>KERUPUK EMPING</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F68" t="inlineStr"/>
+        <v>5000</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>EMPING</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
@@ -2558,7 +2642,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>EMPING</t>
+          <t>KERUPUK MAWAR</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -2583,12 +2667,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>MINUMAN</t>
+          <t>KERUPUK</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ES TEH MANIS</t>
+          <t>KERIPIK TEMPE KOIN PEDES ASIN</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -2596,13 +2680,13 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>ES TEH</t>
+          <t>KERIPIK TEMPE PEDES</t>
         </is>
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>🧊</t>
+          <t>🍘</t>
         </is>
       </c>
     </row>
@@ -2617,12 +2701,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>MINUMAN</t>
+          <t>KERUPUK</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>TEH HANGAT</t>
+          <t>KERIPIK TEMPE KOIN ORI</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -2630,13 +2714,13 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>TEH PANAS</t>
+          <t>KERIPIK TEMPE ORI</t>
         </is>
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>☕</t>
+          <t>🍘</t>
         </is>
       </c>
     </row>
@@ -2656,17 +2740,21 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>ES JERUK</t>
+          <t>MINERAL 500ML</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F72" t="inlineStr"/>
+        <v>2000</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>AIR MINERAL,AIR PUTIH</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>🍊</t>
+          <t>💧</t>
         </is>
       </c>
     </row>
@@ -2686,21 +2774,21 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>JERUK HANGAT</t>
+          <t>MINERAL 1.5L</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>7000</v>
+        <v>3000</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>JERUK PANAS</t>
+          <t>AIR MINERAL BESAR</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>🍊</t>
+          <t>💧</t>
         </is>
       </c>
     </row>
@@ -2720,17 +2808,17 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>ES SUSU</t>
+          <t>LIANG TEH PANDA</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>8000</v>
+        <v>3000</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>🥛</t>
+          <t>🧊</t>
         </is>
       </c>
     </row>
@@ -2750,11 +2838,11 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>KOPI HITAM</t>
+          <t>GOLDA DOLCE LATTE</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
@@ -2780,11 +2868,11 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>KOPI SUSU</t>
+          <t>GOLDA CAPPUCINO</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>8000</v>
+        <v>4000</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
@@ -2810,17 +2898,17 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ES KOPI SUSU</t>
+          <t>TEH BOTOL</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>☕</t>
+          <t>🧊</t>
         </is>
       </c>
     </row>
@@ -2840,21 +2928,17 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>AIR MINERAL</t>
+          <t>AW</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>AIR PUTIH</t>
-        </is>
-      </c>
+        <v>5000</v>
+      </c>
+      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>💧</t>
+          <t>🧊</t>
         </is>
       </c>
     </row>
@@ -2874,13 +2958,17 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>ES CAMPUR</t>
+          <t>TEH PUCUK 500ML</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F79" t="inlineStr"/>
+        <v>5000</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>TEH PUCUK</t>
+        </is>
+      </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
@@ -2904,13 +2992,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>ES TELER</t>
+          <t>POCARI SWEAT</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F80" t="inlineStr"/>
+        <v>5000</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>POCARI</t>
+        </is>
+      </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
@@ -2929,22 +3021,26 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>MINUMAN</t>
+          <t>ROKOK CUKAI</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>JUS ALPUKAT</t>
+          <t>GG FILTER</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F81" t="inlineStr"/>
+        <v>15000</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>GUDANG GARAM FILTER</t>
+        </is>
+      </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>🥑</t>
+          <t>🚬</t>
         </is>
       </c>
     </row>
@@ -2959,22 +3055,26 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>MINUMAN</t>
+          <t>ROKOK CUKAI</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>JUS MANGGA</t>
+          <t>SAMPOERNA MILD</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F82" t="inlineStr"/>
+        <v>17000</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>A MILD</t>
+        </is>
+      </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>🥭</t>
+          <t>🚬</t>
         </is>
       </c>
     </row>
@@ -2989,22 +3089,26 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>MINUMAN</t>
+          <t>ROKOK CUKAI</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>JUS JERUK</t>
+          <t>SURYA 16</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F83" t="inlineStr"/>
+        <v>17000</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>GG SURYA 16</t>
+        </is>
+      </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>🍊</t>
+          <t>🚬</t>
         </is>
       </c>
     </row>
@@ -3024,15 +3128,15 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>GUDANG GARAM SURYA</t>
+          <t>MARLONG</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>25000</v>
+        <v>20000</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>GG SURYA</t>
+          <t>MARLBORO LONG</t>
         </is>
       </c>
       <c r="G84" t="inlineStr"/>
@@ -3053,20 +3157,20 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ROKOK CUKAI</t>
+          <t>ROKOK LOKAL</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>GUDANG GARAM MERAH</t>
+          <t>LA BOLD ITEM 20</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>GG MERAH</t>
+          <t>LA BOLD</t>
         </is>
       </c>
       <c r="G85" t="inlineStr"/>
@@ -3087,16 +3191,16 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ROKOK CUKAI</t>
+          <t>ROKOK LOKAL</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>DJARUM SUPER</t>
+          <t>BLACK MILD</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>22000</v>
+        <v>8000</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
@@ -3117,22 +3221,18 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ROKOK CUKAI</t>
+          <t>ROKOK LOKAL</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>SAMPOERNA MILD</t>
+          <t>LA MANGOBOOST</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>A MILD</t>
-        </is>
-      </c>
+        <v>10000</v>
+      </c>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
@@ -3151,16 +3251,16 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ROKOK CUKAI</t>
+          <t>ROKOK LOKAL</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>MARLBORO</t>
+          <t>LA PURPLEBOOST</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
@@ -3181,16 +3281,16 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ROKOK CUKAI</t>
+          <t>ROKOK LOKAL</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>SURYA PRO MILD</t>
+          <t>MARLBORO VISTA</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
@@ -3216,17 +3316,13 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>L.A BOLD</t>
+          <t>VISTA FORESTFUSION</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>LA BOLD</t>
-        </is>
-      </c>
+        <v>8000</v>
+      </c>
+      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
@@ -3250,11 +3346,11 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>ESSE</t>
+          <t>MARLBORO MERAH</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>15000</v>
+        <v>8000</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
@@ -3280,11 +3376,11 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>MAGNUM</t>
+          <t>ORIS</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>12000</v>
+        <v>6000</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
@@ -3310,7 +3406,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>GUDANG BARU</t>
+          <t>ESSE CHANGE BLUE</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -3340,7 +3436,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>WIN</t>
+          <t>ESSE DOUBLE CLICK</t>
         </is>
       </c>
       <c r="E94" t="n">

</xml_diff>

<commit_message>
Fix menu: hapus + dari nama menu, pindah ke alias
Parser punya combo-splitter yang memecah tanda + jadi 2 item
terpisah (mis. "Soto Daging + Nasi" → "Soto Daging" + "Nasi").
Fix: nama menu pakai spasi (SOTO DAGING NASI), versi dengan +
ditaruh di alias supaya tetap bisa dikenali.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/menu.xlsx
+++ b/data/menu.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KALASAN DADA+NASI</t>
+          <t>KALASAN DADA NASI</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -786,7 +786,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>KALASAN DADA NASI</t>
+          <t>KALASAN DADA+NASI</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -812,7 +812,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KALASAN PAHA+NASI</t>
+          <t>KALASAN PAHA NASI</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>KALASAN PAHA NASI</t>
+          <t>KALASAN PAHA+NASI</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -914,7 +914,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>KUNING DADA+NASI</t>
+          <t>KUNING DADA NASI</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -922,7 +922,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>KUNING DADA NASI</t>
+          <t>KUNING DADA+NASI</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -948,7 +948,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KUNING PAHA+NASI</t>
+          <t>KUNING PAHA NASI</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -956,7 +956,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>KUNING PAHA NASI</t>
+          <t>KUNING PAHA+NASI</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>NASI CHARSIU</t>
+          <t>NASI CHARSIU,CHARSIU AYAM</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>SOTO DAGING+NASI</t>
+          <t>SOTO DAGING NASI</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>SOTO DAGING NASI</t>
+          <t>SOTO DAGING+NASI</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SOTO TETELAN+NASI</t>
+          <t>SOTO TETELAN NASI</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>SOTO TETELAN NASI</t>
+          <t>SOTO TETELAN+NASI</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SOTO AYAM+NASI</t>
+          <t>SOTO AYAM NASI</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SOTO AYAM NASI</t>
+          <t>SOTO AYAM+NASI</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SOP DAGING+NASI</t>
+          <t>SOP DAGING NASI</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SOP DAGING NASI</t>
+          <t>SOP DAGING+NASI</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SOP TETELAN+NASI</t>
+          <t>SOP TETELAN NASI</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>SOP TETELAN NASI</t>
+          <t>SOP TETELAN+NASI</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SOP AYAM+NASI</t>
+          <t>SOP AYAM NASI</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>SOP AYAM NASI</t>
+          <t>SOP AYAM+NASI</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>BASO RACIK MIE+BIHUN</t>
+          <t>BASO RACIK MIE BIHUN</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>BASO RACIK MIE BIHUN,BAKSO RACIK</t>
+          <t>BASO RACIK MIE+BIHUN,BAKSO RACIK</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>

</xml_diff>

<commit_message>
Tambah 73 menu baru (BAKMIE/BIHUN/KWETIAU/NASI CAMPUR/KUAH/toping)
Menu ditambahkan sesuai list Madam Lily:
- BAKMIE (NON HALAL) 10 item — biasa, special, cincang, merah, panggang
- BAKMI PANGSIT 1 item
- MIYABI (MIE AYAM+BABI) 3 varian
- BAKMIE (HALAL) 4 item — ayam kampoeng & kecap
- BIHUN (NON HALAL) 5 item
- KWETIAU (NON HALAL) 9 item
- KWETIAU (HALAL) 2 item
- NASI (HALAL) 1 item
- NASI CAMPUR (NON HALAL) 8 item
- KUAH (NON HALAL) 11 item — bakut, baso, pangsit, kari
- KUAH (HALAL) 7 item — kari ayam, kari sapi, baso gepeng
- TOPING TAMBAHAN 10 item
- MINUMAN: BADAK & SONKIT

Naming convention:
- + dan (JUMBO) di nama diganti spasi/kata biasa
  (contoh: 'BAKMIE BIASA JUMBO' bukan 'BAKMIE BIASA (JUMBO)')
- Versi asli dengan +/() masuk kolom Alias supaya bot Telegram tetap
  bisa parse pesanan yang pakai format asli

Emoji fix:
- 2 item TEMPE/TAHU KUNING yang belum ada emoji → 🌱
- 9 item MINUMAN diseragamkan ke 🥤

Total menu: 166 (dari 93)
</commit_message>
<xml_diff>
--- a/data/menu.xlsx
+++ b/data/menu.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,6 @@
           <t>BUBUR AYAM</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>🥡</t>
@@ -544,8 +543,6 @@
       <c r="E3" t="n">
         <v>12000</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>🥡</t>
@@ -574,8 +571,6 @@
       <c r="E4" t="n">
         <v>2000</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -604,8 +599,6 @@
       <c r="E5" t="n">
         <v>3000</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -634,8 +627,6 @@
       <c r="E6" t="n">
         <v>3000</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -664,8 +655,6 @@
       <c r="E7" t="n">
         <v>3000</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -694,8 +683,6 @@
       <c r="E8" t="n">
         <v>3000</v>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -724,8 +711,6 @@
       <c r="E9" t="n">
         <v>3000</v>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -754,8 +739,6 @@
       <c r="E10" t="n">
         <v>3000</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -789,7 +772,6 @@
           <t>KALASAN DADA+NASI</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -823,7 +805,6 @@
           <t>KALASAN PAHA+NASI</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -852,7 +833,6 @@
       <c r="E13" t="n">
         <v>10000</v>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -886,7 +866,6 @@
       <c r="E14" t="n">
         <v>10000</v>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -925,7 +904,6 @@
           <t>KUNING DADA+NASI</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -959,7 +937,6 @@
           <t>KUNING PAHA+NASI</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -988,7 +965,6 @@
       <c r="E17" t="n">
         <v>10000</v>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1022,7 +998,6 @@
       <c r="E18" t="n">
         <v>10000</v>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1056,13 +1031,16 @@
       <c r="E19" t="n">
         <v>2000</v>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>tambahan</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>🌱</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1086,13 +1064,16 @@
       <c r="E20" t="n">
         <v>2000</v>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>tambahan</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>🌱</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1121,7 +1102,6 @@
           <t>PENYET CABE IJO</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -1155,7 +1135,6 @@
           <t>NASI CHARSIU,CHARSIU AYAM</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>🌚</t>
@@ -1189,7 +1168,6 @@
           <t>AYAM SEREH</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -1223,7 +1201,6 @@
           <t>SOTO DAGING+NASI</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1257,7 +1234,6 @@
           <t>SOTO TETELAN+NASI</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1291,7 +1267,6 @@
           <t>SOTO AYAM+NASI</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1325,7 +1300,6 @@
           <t>SOP DAGING+NASI</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1359,7 +1333,6 @@
           <t>SOP TETELAN+NASI</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1393,7 +1366,6 @@
           <t>SOP AYAM+NASI</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1422,7 +1394,6 @@
       <c r="E30" t="n">
         <v>12000</v>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1456,7 +1427,6 @@
       <c r="E31" t="n">
         <v>10000</v>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1490,7 +1460,6 @@
       <c r="E32" t="n">
         <v>12000</v>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1524,7 +1493,6 @@
       <c r="E33" t="n">
         <v>12000</v>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1558,7 +1526,6 @@
       <c r="E34" t="n">
         <v>10000</v>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1592,7 +1559,6 @@
       <c r="E35" t="n">
         <v>12000</v>
       </c>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1631,7 +1597,6 @@
           <t>BASO RACIK MIE+BIHUN,BAKSO RACIK</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>🍥</t>
@@ -1665,7 +1630,6 @@
           <t>BAKSO RACIK NASI</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>🍥</t>
@@ -1699,7 +1663,6 @@
           <t>NASKU</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>🥚</t>
@@ -1728,8 +1691,6 @@
       <c r="E39" t="n">
         <v>12000</v>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>🥚</t>
@@ -1763,7 +1724,6 @@
           <t>NASKU KALASAN</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>🥚</t>
@@ -1797,7 +1757,6 @@
           <t>NASKU KUNING</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>🥚</t>
@@ -1826,8 +1785,6 @@
       <c r="E42" t="n">
         <v>7000</v>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>🍚</t>
@@ -1856,8 +1813,6 @@
       <c r="E43" t="n">
         <v>12000</v>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>🍚</t>
@@ -1886,8 +1841,6 @@
       <c r="E44" t="n">
         <v>15000</v>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>🍚</t>
@@ -1916,8 +1869,6 @@
       <c r="E45" t="n">
         <v>15000</v>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>🍚</t>
@@ -1946,8 +1897,6 @@
       <c r="E46" t="n">
         <v>1000</v>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -1976,8 +1925,6 @@
       <c r="E47" t="n">
         <v>1000</v>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2006,8 +1953,6 @@
       <c r="E48" t="n">
         <v>3000</v>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2036,8 +1981,6 @@
       <c r="E49" t="n">
         <v>3000</v>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2066,8 +2009,6 @@
       <c r="E50" t="n">
         <v>3000</v>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2101,7 +2042,6 @@
           <t>PISANG COKLAT</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>🍫</t>
@@ -2130,8 +2070,6 @@
       <c r="E52" t="n">
         <v>5000</v>
       </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2160,8 +2098,6 @@
       <c r="E53" t="n">
         <v>5000</v>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2190,8 +2126,6 @@
       <c r="E54" t="n">
         <v>5000</v>
       </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2220,8 +2154,6 @@
       <c r="E55" t="n">
         <v>5000</v>
       </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2250,8 +2182,6 @@
       <c r="E56" t="n">
         <v>5000</v>
       </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2280,8 +2210,6 @@
       <c r="E57" t="n">
         <v>5000</v>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2310,8 +2238,6 @@
       <c r="E58" t="n">
         <v>5000</v>
       </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2340,8 +2266,6 @@
       <c r="E59" t="n">
         <v>5000</v>
       </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2370,8 +2294,6 @@
       <c r="E60" t="n">
         <v>5000</v>
       </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2400,8 +2322,6 @@
       <c r="E61" t="n">
         <v>5000</v>
       </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2435,7 +2355,6 @@
           <t>BUBUR KACANG IJO</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2464,8 +2383,6 @@
       <c r="E63" t="n">
         <v>5000</v>
       </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2494,8 +2411,6 @@
       <c r="E64" t="n">
         <v>5000</v>
       </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>🍮</t>
@@ -2524,8 +2439,6 @@
       <c r="E65" t="n">
         <v>5000</v>
       </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2554,8 +2467,6 @@
       <c r="E66" t="n">
         <v>5000</v>
       </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>🦐</t>
@@ -2584,8 +2495,6 @@
       <c r="E67" t="n">
         <v>5000</v>
       </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2619,7 +2528,6 @@
           <t>EMPING</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2648,8 +2556,6 @@
       <c r="E69" t="n">
         <v>5000</v>
       </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2683,7 +2589,6 @@
           <t>KERIPIK TEMPE PEDES</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2717,7 +2622,6 @@
           <t>KERIPIK TEMPE ORI</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2751,10 +2655,9 @@
           <t>AIR MINERAL,AIR PUTIH</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>💧</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -2785,10 +2688,9 @@
           <t>AIR MINERAL BESAR</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>💧</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -2814,11 +2716,9 @@
       <c r="E74" t="n">
         <v>3000</v>
       </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>🧊</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -2844,11 +2744,9 @@
       <c r="E75" t="n">
         <v>4000</v>
       </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>☕</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -2874,11 +2772,9 @@
       <c r="E76" t="n">
         <v>4000</v>
       </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>☕</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -2904,11 +2800,9 @@
       <c r="E77" t="n">
         <v>4000</v>
       </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>🧊</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -2934,11 +2828,9 @@
       <c r="E78" t="n">
         <v>5000</v>
       </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>🧊</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -2969,10 +2861,9 @@
           <t>TEH PUCUK</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>🧊</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -3003,10 +2894,9 @@
           <t>POCARI</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>🧊</t>
+          <t>🥤</t>
         </is>
       </c>
     </row>
@@ -3037,7 +2927,6 @@
           <t>GUDANG GARAM FILTER</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3071,7 +2960,6 @@
           <t>A MILD</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3105,7 +2993,6 @@
           <t>GG SURYA 16</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3139,7 +3026,6 @@
           <t>MARLBORO LONG</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3173,7 +3059,6 @@
           <t>LA BOLD</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3202,8 +3087,6 @@
       <c r="E86" t="n">
         <v>8000</v>
       </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3232,8 +3115,6 @@
       <c r="E87" t="n">
         <v>10000</v>
       </c>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3262,8 +3143,6 @@
       <c r="E88" t="n">
         <v>10000</v>
       </c>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3292,8 +3171,6 @@
       <c r="E89" t="n">
         <v>8000</v>
       </c>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3322,8 +3199,6 @@
       <c r="E90" t="n">
         <v>8000</v>
       </c>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3352,8 +3227,6 @@
       <c r="E91" t="n">
         <v>8000</v>
       </c>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3382,8 +3255,6 @@
       <c r="E92" t="n">
         <v>6000</v>
       </c>
-      <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3412,8 +3283,6 @@
       <c r="E93" t="n">
         <v>8000</v>
       </c>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3442,11 +3311,2248 @@
       <c r="E94" t="n">
         <v>8000</v>
       </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>🚬</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>BAKMIE BIASA</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>BAKMIE BIASA JUMBO</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>BAKMIE BIASA (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>BAKMIE SPECIAL</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>22000</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>BAKMIE SPECIAL JUMBO</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>27000</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>BAKMIE SPECIAL (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>BAKMIE BABI CINCANG</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>BAKMIE BABI CINCANG JUMBO</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>BAKMI BABI CINCANG (JUMBO), BAKMIE BABI CINCANG (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>BAKMIE BABI MERAH</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>BAKMIE BABI MERAH JUMBO</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>BAKMIE BABI MERAH (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>BAKMIE BABI PANGGANG</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>BAKMIE (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>BAKMIE BABI PANGGANG JUMBO</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>BAKMI BABI PANGGANG (JUMBO), BAKMIE BABI PANGGANG (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>BAKMI PANGSIT</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>BAKMI PANGSIT ISTIMEWA</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>22000</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>MIYABI (MIE AYAM+BABI)</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>BAKMI AYAM KAMPOENG BABI CINCANG</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>BAKMI AYAM KAMPOENG+B.CINCANG, MIYABI CINCANG</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>MIYABI (MIE AYAM+BABI)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>BAKMI AYAM KAMPOENG BABI MERAH</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>BAKMI AYAM KAMPOENG+B.MERAH, MIYABI MERAH</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>MIYABI (MIE AYAM+BABI)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>BAKMI AYAM KAMPOENG BABI PANGGANG</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>BAKMI AYAM KAMPOENG+B.PANGGANG, MIYABI PANGGANG</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>BAKMIE (HALAL)</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>BAKMIE AYAM KAMPOENG</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>BAKMIE (HALAL)</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>BAKMIE AYAM KAMPOENG JUMBO</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>23000</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>BAKMIE AYAM KAMPOENG (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>BAKMIE (HALAL)</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>BAKMIE AYAM KECAP</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>BAKMIE (HALAL)</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>BAKMIE AYAM KECAP JUMBO</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>BAKMIE AYAM KECAP (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>BIHUN (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>BIHUN BIASA</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>BIHUN (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>BIHUN BABI CINCANG</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>BIHUN (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>BIHUN BABI PANGGANG</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>BIHUN (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>BIHUN BABI MERAH</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>BIHUN (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>BIHUN PANGSIT ISTIMEWA</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>22000</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>KWETIAU BIASA</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>KWETIAU BIASA JUMBO</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>KWETIAU BIASA (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI CINCANG</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI CINCANG JUMBO</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI CINCANG (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI MERAH</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI MERAH BIASA</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI MERAH JUMBO</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI MERAH (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI PANGGANG</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI PANGGANG JUMBO</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>KWETIAU BABI PANGGANG (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>KWETIAU (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>KWETIAU PANGSIT ISTIMEWA</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>22000</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>KWETIAU (HALAL)</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>KWETIAU AYAM KAMPOENG</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>KWETIAU (HALAL)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>KWETIAU AYAM KAMPOENG JUMBO</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>23000</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>🍜</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>NASI (HALAL)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>NASI AYAM PACAMKE</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>🐓</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>17000</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>🐷</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR JUMBO</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>28000</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>🐷</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>NASI BABI PANGGANG</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>23000</v>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>🐷</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>NASI BABI PANGGANG JUMBO</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>28000</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>NASI BABI PANGGANG (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>🐷</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>NASI BABI MERAH</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>17000</v>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>🐷</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>NASI BABI MERAH JUMBO</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>NASI BABI MERAH (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>🐷</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>NASI BABI KECAP</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>17000</v>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>🐷</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>NASI CAMPUR (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>NASI BABI KECAP JUMBO</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>NASI BABI KECAP (JUMBO)</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>🐷</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>BAKUT TEH NASI</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>21000</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>BAKUT TEH + NASI</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>BAKUT TEH TANPA NASI</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>19000</v>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>BAKUT SAYUR ASIN NASI</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>21000</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>BAKUT SAYUR ASIN + NASI</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>BAKUT SAYUR ASIN TANPA NASI</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>19000</v>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>BASO BABI NASI</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>BASO BABI + NASI</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>BASO BABI TANPA NASI</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>PANGSIT REBUS NASI</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>PANGSIT REBUS + NASI (ISI 6PCS)</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>PANGSIT REBUS TANPA NASI</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>PANGSIT REBUS TANPA NASI (ISI 6PCS)</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>KARI BABI PANGGANG NASI</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>23000</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>KARI BABI PANGGANG + NASI</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>🍛</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>KARI BIHUN BABI PANGGANG</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>23000</v>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>🍛</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>KUAH (NON HALAL)</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>KARI BIHUN BABI PANGGANG NASI</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>26000</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>KARI BIHUN BABI PANGGANG + NASI</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>🍛</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>KUAH (HALAL)</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>KARI AYAM NASI</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>KARI AYAM + NASI</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>🍛</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>KUAH (HALAL)</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>KARI AYAM TANPA NASI</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>🍛</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>KUAH (HALAL)</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>KARI DAGING SAPI NASI</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>17000</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>KARI DAGING SAPI + NASI</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>🍛</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>KUAH (HALAL)</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>KARI DAGING SAPI BIHUN</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>17000</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>KARI DAGING SAPI + BIHUN</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>🍛</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>KUAH (HALAL)</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>KARI DAGING SAPI NASI BIHUN</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>KARI DAGING SAPI + NASI + BIHUN</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>🍛</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>KUAH (HALAL)</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>BASO GEPENG NASI</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>BASO GEPENG + NASI</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>KUAH (HALAL)</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>BASO GEPENG TANPA NASI</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>🍲</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>NASI PUTIH</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>🍚</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>BABI PANGGANG 100GR</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>23000</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>BABI PANGGANG (100GR)</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>🥓</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>BABI MERAH 100GR</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>17000</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>BABI MERAH (100GR)</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>🥓</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>PANGSIT GORENG</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>PANGSIT GORENG (ISI 3)</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>🥟</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>BASO BABI GORENG</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>BASO BABI GORENG (2PCS)</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>🥟</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>BASO AYAM GORENG</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>BASO AYAM GORENG (2PCS)</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>🥟</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>TELUR KECAP</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>🥚</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>KERUPUK UDANG TOPING</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>KERUPUK UDANG</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>🍘</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>KERUPUK PUTIH TOPING</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>KERUPUK PUTIH</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>🍘</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>TOPING TAMBAHAN</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>EMPING TOPING</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>EMPING</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>🍘</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>MINUMAN</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>BADAK</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>🥤</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>MADAM LILY</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>MINUMAN</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>SONKIT</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>6000</v>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>🥤</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Tambah 73 menu baru (BAKMIE/BIHUN/KWETIAU/NASI CAMPUR/KUAH/toping)"
This reverts commit 8e314af85cf2d168623376a39d305da02a0dd9c1.
</commit_message>
<xml_diff>
--- a/data/menu.xlsx
+++ b/data/menu.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H167"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -515,6 +515,7 @@
           <t>BUBUR AYAM</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>🥡</t>
@@ -543,6 +544,8 @@
       <c r="E3" t="n">
         <v>12000</v>
       </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>🥡</t>
@@ -571,6 +574,8 @@
       <c r="E4" t="n">
         <v>2000</v>
       </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -599,6 +604,8 @@
       <c r="E5" t="n">
         <v>3000</v>
       </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -627,6 +634,8 @@
       <c r="E6" t="n">
         <v>3000</v>
       </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -655,6 +664,8 @@
       <c r="E7" t="n">
         <v>3000</v>
       </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -683,6 +694,8 @@
       <c r="E8" t="n">
         <v>3000</v>
       </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -711,6 +724,8 @@
       <c r="E9" t="n">
         <v>3000</v>
       </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -739,6 +754,8 @@
       <c r="E10" t="n">
         <v>3000</v>
       </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -772,6 +789,7 @@
           <t>KALASAN DADA+NASI</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -805,6 +823,7 @@
           <t>KALASAN PAHA+NASI</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -833,6 +852,7 @@
       <c r="E13" t="n">
         <v>10000</v>
       </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -866,6 +886,7 @@
       <c r="E14" t="n">
         <v>10000</v>
       </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -904,6 +925,7 @@
           <t>KUNING DADA+NASI</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -937,6 +959,7 @@
           <t>KUNING PAHA+NASI</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -965,6 +988,7 @@
       <c r="E17" t="n">
         <v>10000</v>
       </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -998,6 +1022,7 @@
       <c r="E18" t="n">
         <v>10000</v>
       </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1031,16 +1056,13 @@
       <c r="E19" t="n">
         <v>2000</v>
       </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>tambahan</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>🌱</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1064,16 +1086,13 @@
       <c r="E20" t="n">
         <v>2000</v>
       </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>tambahan</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>🌱</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1102,6 +1121,7 @@
           <t>PENYET CABE IJO</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -1135,6 +1155,7 @@
           <t>NASI CHARSIU,CHARSIU AYAM</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>🌚</t>
@@ -1168,6 +1189,7 @@
           <t>AYAM SEREH</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>🍗</t>
@@ -1201,6 +1223,7 @@
           <t>SOTO DAGING+NASI</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1234,6 +1257,7 @@
           <t>SOTO TETELAN+NASI</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1267,6 +1291,7 @@
           <t>SOTO AYAM+NASI</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1300,6 +1325,7 @@
           <t>SOP DAGING+NASI</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1333,6 +1359,7 @@
           <t>SOP TETELAN+NASI</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1366,6 +1393,7 @@
           <t>SOP AYAM+NASI</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>🍲</t>
@@ -1394,6 +1422,7 @@
       <c r="E30" t="n">
         <v>12000</v>
       </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1427,6 +1456,7 @@
       <c r="E31" t="n">
         <v>10000</v>
       </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1460,6 +1490,7 @@
       <c r="E32" t="n">
         <v>12000</v>
       </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1493,6 +1524,7 @@
       <c r="E33" t="n">
         <v>12000</v>
       </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1526,6 +1558,7 @@
       <c r="E34" t="n">
         <v>10000</v>
       </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1559,6 +1592,7 @@
       <c r="E35" t="n">
         <v>12000</v>
       </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>tanpa nasi</t>
@@ -1597,6 +1631,7 @@
           <t>BASO RACIK MIE+BIHUN,BAKSO RACIK</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>🍥</t>
@@ -1630,6 +1665,7 @@
           <t>BAKSO RACIK NASI</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>🍥</t>
@@ -1663,6 +1699,7 @@
           <t>NASKU</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>🥚</t>
@@ -1691,6 +1728,8 @@
       <c r="E39" t="n">
         <v>12000</v>
       </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>🥚</t>
@@ -1724,6 +1763,7 @@
           <t>NASKU KALASAN</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>🥚</t>
@@ -1757,6 +1797,7 @@
           <t>NASKU KUNING</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>🥚</t>
@@ -1785,6 +1826,8 @@
       <c r="E42" t="n">
         <v>7000</v>
       </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>🍚</t>
@@ -1813,6 +1856,8 @@
       <c r="E43" t="n">
         <v>12000</v>
       </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>🍚</t>
@@ -1841,6 +1886,8 @@
       <c r="E44" t="n">
         <v>15000</v>
       </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>🍚</t>
@@ -1869,6 +1916,8 @@
       <c r="E45" t="n">
         <v>15000</v>
       </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>🍚</t>
@@ -1897,6 +1946,8 @@
       <c r="E46" t="n">
         <v>1000</v>
       </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -1925,6 +1976,8 @@
       <c r="E47" t="n">
         <v>1000</v>
       </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -1953,6 +2006,8 @@
       <c r="E48" t="n">
         <v>3000</v>
       </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -1981,6 +2036,8 @@
       <c r="E49" t="n">
         <v>3000</v>
       </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2009,6 +2066,8 @@
       <c r="E50" t="n">
         <v>3000</v>
       </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2042,6 +2101,7 @@
           <t>PISANG COKLAT</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>🍫</t>
@@ -2070,6 +2130,8 @@
       <c r="E52" t="n">
         <v>5000</v>
       </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2098,6 +2160,8 @@
       <c r="E53" t="n">
         <v>5000</v>
       </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2126,6 +2190,8 @@
       <c r="E54" t="n">
         <v>5000</v>
       </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2154,6 +2220,8 @@
       <c r="E55" t="n">
         <v>5000</v>
       </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2182,6 +2250,8 @@
       <c r="E56" t="n">
         <v>5000</v>
       </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2210,6 +2280,8 @@
       <c r="E57" t="n">
         <v>5000</v>
       </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2238,6 +2310,8 @@
       <c r="E58" t="n">
         <v>5000</v>
       </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2266,6 +2340,8 @@
       <c r="E59" t="n">
         <v>5000</v>
       </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2294,6 +2370,8 @@
       <c r="E60" t="n">
         <v>5000</v>
       </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2322,6 +2400,8 @@
       <c r="E61" t="n">
         <v>5000</v>
       </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2355,6 +2435,7 @@
           <t>BUBUR KACANG IJO</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2383,6 +2464,8 @@
       <c r="E63" t="n">
         <v>5000</v>
       </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>🍢</t>
@@ -2411,6 +2494,8 @@
       <c r="E64" t="n">
         <v>5000</v>
       </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>🍮</t>
@@ -2439,6 +2524,8 @@
       <c r="E65" t="n">
         <v>5000</v>
       </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2467,6 +2554,8 @@
       <c r="E66" t="n">
         <v>5000</v>
       </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>🦐</t>
@@ -2495,6 +2584,8 @@
       <c r="E67" t="n">
         <v>5000</v>
       </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2528,6 +2619,7 @@
           <t>EMPING</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2556,6 +2648,8 @@
       <c r="E69" t="n">
         <v>5000</v>
       </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2589,6 +2683,7 @@
           <t>KERIPIK TEMPE PEDES</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2622,6 +2717,7 @@
           <t>KERIPIK TEMPE ORI</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>🍘</t>
@@ -2655,9 +2751,10 @@
           <t>AIR MINERAL,AIR PUTIH</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>💧</t>
         </is>
       </c>
     </row>
@@ -2688,9 +2785,10 @@
           <t>AIR MINERAL BESAR</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>💧</t>
         </is>
       </c>
     </row>
@@ -2716,9 +2814,11 @@
       <c r="E74" t="n">
         <v>3000</v>
       </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>🧊</t>
         </is>
       </c>
     </row>
@@ -2744,9 +2844,11 @@
       <c r="E75" t="n">
         <v>4000</v>
       </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>☕</t>
         </is>
       </c>
     </row>
@@ -2772,9 +2874,11 @@
       <c r="E76" t="n">
         <v>4000</v>
       </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>☕</t>
         </is>
       </c>
     </row>
@@ -2800,9 +2904,11 @@
       <c r="E77" t="n">
         <v>4000</v>
       </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>🧊</t>
         </is>
       </c>
     </row>
@@ -2828,9 +2934,11 @@
       <c r="E78" t="n">
         <v>5000</v>
       </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>🧊</t>
         </is>
       </c>
     </row>
@@ -2861,9 +2969,10 @@
           <t>TEH PUCUK</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>🧊</t>
         </is>
       </c>
     </row>
@@ -2894,9 +3003,10 @@
           <t>POCARI</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>🥤</t>
+          <t>🧊</t>
         </is>
       </c>
     </row>
@@ -2927,6 +3037,7 @@
           <t>GUDANG GARAM FILTER</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -2960,6 +3071,7 @@
           <t>A MILD</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -2993,6 +3105,7 @@
           <t>GG SURYA 16</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3026,6 +3139,7 @@
           <t>MARLBORO LONG</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3059,6 +3173,7 @@
           <t>LA BOLD</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3087,6 +3202,8 @@
       <c r="E86" t="n">
         <v>8000</v>
       </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3115,6 +3232,8 @@
       <c r="E87" t="n">
         <v>10000</v>
       </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3143,6 +3262,8 @@
       <c r="E88" t="n">
         <v>10000</v>
       </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3171,6 +3292,8 @@
       <c r="E89" t="n">
         <v>8000</v>
       </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3199,6 +3322,8 @@
       <c r="E90" t="n">
         <v>8000</v>
       </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3227,6 +3352,8 @@
       <c r="E91" t="n">
         <v>8000</v>
       </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3255,6 +3382,8 @@
       <c r="E92" t="n">
         <v>6000</v>
       </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3283,6 +3412,8 @@
       <c r="E93" t="n">
         <v>8000</v>
       </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>🚬</t>
@@ -3311,2248 +3442,11 @@
       <c r="E94" t="n">
         <v>8000</v>
       </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>🚬</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n">
-        <v>94</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>BAKMIE BIASA</t>
-        </is>
-      </c>
-      <c r="E95" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>95</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>BAKMIE BIASA JUMBO</t>
-        </is>
-      </c>
-      <c r="E96" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>BAKMIE BIASA (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>96</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>BAKMIE SPECIAL</t>
-        </is>
-      </c>
-      <c r="E97" t="n">
-        <v>22000</v>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>97</v>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>BAKMIE SPECIAL JUMBO</t>
-        </is>
-      </c>
-      <c r="E98" t="n">
-        <v>27000</v>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>BAKMIE SPECIAL (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>BAKMIE BABI CINCANG</t>
-        </is>
-      </c>
-      <c r="E99" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>99</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>BAKMIE BABI CINCANG JUMBO</t>
-        </is>
-      </c>
-      <c r="E100" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>BAKMI BABI CINCANG (JUMBO), BAKMIE BABI CINCANG (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>100</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>BAKMIE BABI MERAH</t>
-        </is>
-      </c>
-      <c r="E101" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
-        <v>101</v>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>BAKMIE BABI MERAH JUMBO</t>
-        </is>
-      </c>
-      <c r="E102" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>BAKMIE BABI MERAH (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
-        <v>102</v>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>BAKMIE BABI PANGGANG</t>
-        </is>
-      </c>
-      <c r="E103" t="n">
-        <v>20000</v>
-      </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
-        <v>103</v>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>BAKMIE (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>BAKMIE BABI PANGGANG JUMBO</t>
-        </is>
-      </c>
-      <c r="E104" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>BAKMI BABI PANGGANG (JUMBO), BAKMIE BABI PANGGANG (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
-        <v>104</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>BAKMI PANGSIT</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>BAKMI PANGSIT ISTIMEWA</t>
-        </is>
-      </c>
-      <c r="E105" t="n">
-        <v>22000</v>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
-        <v>105</v>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>MIYABI (MIE AYAM+BABI)</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>BAKMI AYAM KAMPOENG BABI CINCANG</t>
-        </is>
-      </c>
-      <c r="E106" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>BAKMI AYAM KAMPOENG+B.CINCANG, MIYABI CINCANG</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
-        <v>106</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>MIYABI (MIE AYAM+BABI)</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>BAKMI AYAM KAMPOENG BABI MERAH</t>
-        </is>
-      </c>
-      <c r="E107" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>BAKMI AYAM KAMPOENG+B.MERAH, MIYABI MERAH</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
-        <v>107</v>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>MIYABI (MIE AYAM+BABI)</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>BAKMI AYAM KAMPOENG BABI PANGGANG</t>
-        </is>
-      </c>
-      <c r="E108" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>BAKMI AYAM KAMPOENG+B.PANGGANG, MIYABI PANGGANG</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>108</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>BAKMIE (HALAL)</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>BAKMIE AYAM KAMPOENG</t>
-        </is>
-      </c>
-      <c r="E109" t="n">
-        <v>18000</v>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>109</v>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>BAKMIE (HALAL)</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>BAKMIE AYAM KAMPOENG JUMBO</t>
-        </is>
-      </c>
-      <c r="E110" t="n">
-        <v>23000</v>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>BAKMIE AYAM KAMPOENG (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>110</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>BAKMIE (HALAL)</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>BAKMIE AYAM KECAP</t>
-        </is>
-      </c>
-      <c r="E111" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>111</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>BAKMIE (HALAL)</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>BAKMIE AYAM KECAP JUMBO</t>
-        </is>
-      </c>
-      <c r="E112" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>BAKMIE AYAM KECAP (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>112</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>BIHUN (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>BIHUN BIASA</t>
-        </is>
-      </c>
-      <c r="E113" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>113</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>BIHUN (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>BIHUN BABI CINCANG</t>
-        </is>
-      </c>
-      <c r="E114" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>114</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>BIHUN (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>BIHUN BABI PANGGANG</t>
-        </is>
-      </c>
-      <c r="E115" t="n">
-        <v>20000</v>
-      </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>115</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>BIHUN (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>BIHUN BABI MERAH</t>
-        </is>
-      </c>
-      <c r="E116" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
-        <v>116</v>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>BIHUN (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>BIHUN PANGSIT ISTIMEWA</t>
-        </is>
-      </c>
-      <c r="E117" t="n">
-        <v>22000</v>
-      </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
-        <v>117</v>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>KWETIAU BIASA</t>
-        </is>
-      </c>
-      <c r="E118" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
-        <v>118</v>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>KWETIAU BIASA JUMBO</t>
-        </is>
-      </c>
-      <c r="E119" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>KWETIAU BIASA (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>119</v>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI CINCANG</t>
-        </is>
-      </c>
-      <c r="E120" t="n">
-        <v>14000</v>
-      </c>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>120</v>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI CINCANG JUMBO</t>
-        </is>
-      </c>
-      <c r="E121" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI CINCANG (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="n">
-        <v>121</v>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI MERAH</t>
-        </is>
-      </c>
-      <c r="E122" t="n">
-        <v>14000</v>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI MERAH BIASA</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="n">
-        <v>122</v>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI MERAH JUMBO</t>
-        </is>
-      </c>
-      <c r="E123" t="n">
-        <v>19000</v>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI MERAH (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>123</v>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI PANGGANG</t>
-        </is>
-      </c>
-      <c r="E124" t="n">
-        <v>20000</v>
-      </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
-        <v>124</v>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI PANGGANG JUMBO</t>
-        </is>
-      </c>
-      <c r="E125" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>KWETIAU BABI PANGGANG (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
-        <v>125</v>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>KWETIAU (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>KWETIAU PANGSIT ISTIMEWA</t>
-        </is>
-      </c>
-      <c r="E126" t="n">
-        <v>22000</v>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
-        <v>126</v>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>KWETIAU (HALAL)</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>KWETIAU AYAM KAMPOENG</t>
-        </is>
-      </c>
-      <c r="E127" t="n">
-        <v>18000</v>
-      </c>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>127</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>KWETIAU (HALAL)</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>KWETIAU AYAM KAMPOENG JUMBO</t>
-        </is>
-      </c>
-      <c r="E128" t="n">
-        <v>23000</v>
-      </c>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>🍜</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="n">
-        <v>128</v>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>NASI (HALAL)</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>NASI AYAM PACAMKE</t>
-        </is>
-      </c>
-      <c r="E129" t="n">
-        <v>18000</v>
-      </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>🐓</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="n">
-        <v>129</v>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR</t>
-        </is>
-      </c>
-      <c r="E130" t="n">
-        <v>17000</v>
-      </c>
-      <c r="H130" t="inlineStr">
-        <is>
-          <t>🐷</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="n">
-        <v>130</v>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR JUMBO</t>
-        </is>
-      </c>
-      <c r="E131" t="n">
-        <v>28000</v>
-      </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>🐷</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="n">
-        <v>131</v>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>NASI BABI PANGGANG</t>
-        </is>
-      </c>
-      <c r="E132" t="n">
-        <v>23000</v>
-      </c>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t>🐷</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="n">
-        <v>132</v>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>NASI BABI PANGGANG JUMBO</t>
-        </is>
-      </c>
-      <c r="E133" t="n">
-        <v>28000</v>
-      </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>NASI BABI PANGGANG (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t>🐷</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="n">
-        <v>133</v>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>NASI BABI MERAH</t>
-        </is>
-      </c>
-      <c r="E134" t="n">
-        <v>17000</v>
-      </c>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t>🐷</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="n">
-        <v>134</v>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>NASI BABI MERAH JUMBO</t>
-        </is>
-      </c>
-      <c r="E135" t="n">
-        <v>22000</v>
-      </c>
-      <c r="F135" t="inlineStr">
-        <is>
-          <t>NASI BABI MERAH (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H135" t="inlineStr">
-        <is>
-          <t>🐷</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="n">
-        <v>135</v>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>NASI BABI KECAP</t>
-        </is>
-      </c>
-      <c r="E136" t="n">
-        <v>17000</v>
-      </c>
-      <c r="H136" t="inlineStr">
-        <is>
-          <t>🐷</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="n">
-        <v>136</v>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>NASI CAMPUR (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>NASI BABI KECAP JUMBO</t>
-        </is>
-      </c>
-      <c r="E137" t="n">
-        <v>22000</v>
-      </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t>NASI BABI KECAP (JUMBO)</t>
-        </is>
-      </c>
-      <c r="H137" t="inlineStr">
-        <is>
-          <t>🐷</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="n">
-        <v>137</v>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>BAKUT TEH NASI</t>
-        </is>
-      </c>
-      <c r="E138" t="n">
-        <v>21000</v>
-      </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>BAKUT TEH + NASI</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="n">
-        <v>138</v>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>BAKUT TEH TANPA NASI</t>
-        </is>
-      </c>
-      <c r="E139" t="n">
-        <v>19000</v>
-      </c>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="n">
-        <v>139</v>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>BAKUT SAYUR ASIN NASI</t>
-        </is>
-      </c>
-      <c r="E140" t="n">
-        <v>21000</v>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>BAKUT SAYUR ASIN + NASI</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="n">
-        <v>140</v>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>BAKUT SAYUR ASIN TANPA NASI</t>
-        </is>
-      </c>
-      <c r="E141" t="n">
-        <v>19000</v>
-      </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="n">
-        <v>141</v>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>BASO BABI NASI</t>
-        </is>
-      </c>
-      <c r="E142" t="n">
-        <v>14000</v>
-      </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>BASO BABI + NASI</t>
-        </is>
-      </c>
-      <c r="H142" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="n">
-        <v>142</v>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>BASO BABI TANPA NASI</t>
-        </is>
-      </c>
-      <c r="E143" t="n">
-        <v>12000</v>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="n">
-        <v>143</v>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>PANGSIT REBUS NASI</t>
-        </is>
-      </c>
-      <c r="E144" t="n">
-        <v>14000</v>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>PANGSIT REBUS + NASI (ISI 6PCS)</t>
-        </is>
-      </c>
-      <c r="H144" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="n">
-        <v>144</v>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>PANGSIT REBUS TANPA NASI</t>
-        </is>
-      </c>
-      <c r="E145" t="n">
-        <v>12000</v>
-      </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>PANGSIT REBUS TANPA NASI (ISI 6PCS)</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="n">
-        <v>145</v>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>KARI BABI PANGGANG NASI</t>
-        </is>
-      </c>
-      <c r="E146" t="n">
-        <v>23000</v>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>KARI BABI PANGGANG + NASI</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="n">
-        <v>146</v>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>KARI BIHUN BABI PANGGANG</t>
-        </is>
-      </c>
-      <c r="E147" t="n">
-        <v>23000</v>
-      </c>
-      <c r="H147" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="n">
-        <v>147</v>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>KUAH (NON HALAL)</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>KARI BIHUN BABI PANGGANG NASI</t>
-        </is>
-      </c>
-      <c r="E148" t="n">
-        <v>26000</v>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>KARI BIHUN BABI PANGGANG + NASI</t>
-        </is>
-      </c>
-      <c r="H148" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="n">
-        <v>148</v>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>KUAH (HALAL)</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>KARI AYAM NASI</t>
-        </is>
-      </c>
-      <c r="E149" t="n">
-        <v>14000</v>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>KARI AYAM + NASI</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="n">
-        <v>149</v>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>KUAH (HALAL)</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>KARI AYAM TANPA NASI</t>
-        </is>
-      </c>
-      <c r="E150" t="n">
-        <v>12000</v>
-      </c>
-      <c r="H150" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="n">
-        <v>150</v>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>KUAH (HALAL)</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>KARI DAGING SAPI NASI</t>
-        </is>
-      </c>
-      <c r="E151" t="n">
-        <v>17000</v>
-      </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>KARI DAGING SAPI + NASI</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="n">
-        <v>151</v>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>KUAH (HALAL)</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>KARI DAGING SAPI BIHUN</t>
-        </is>
-      </c>
-      <c r="E152" t="n">
-        <v>17000</v>
-      </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>KARI DAGING SAPI + BIHUN</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="n">
-        <v>152</v>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>KUAH (HALAL)</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>KARI DAGING SAPI NASI BIHUN</t>
-        </is>
-      </c>
-      <c r="E153" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>KARI DAGING SAPI + NASI + BIHUN</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>🍛</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="n">
-        <v>153</v>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>KUAH (HALAL)</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>BASO GEPENG NASI</t>
-        </is>
-      </c>
-      <c r="E154" t="n">
-        <v>14000</v>
-      </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>BASO GEPENG + NASI</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="n">
-        <v>154</v>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>KUAH (HALAL)</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>BASO GEPENG TANPA NASI</t>
-        </is>
-      </c>
-      <c r="E155" t="n">
-        <v>12000</v>
-      </c>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>🍲</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="n">
-        <v>155</v>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>NASI PUTIH</t>
-        </is>
-      </c>
-      <c r="E156" t="n">
-        <v>3000</v>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>🍚</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="n">
-        <v>156</v>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>BABI PANGGANG 100GR</t>
-        </is>
-      </c>
-      <c r="E157" t="n">
-        <v>23000</v>
-      </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>BABI PANGGANG (100GR)</t>
-        </is>
-      </c>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t>🥓</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="n">
-        <v>157</v>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>BABI MERAH 100GR</t>
-        </is>
-      </c>
-      <c r="E158" t="n">
-        <v>17000</v>
-      </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>BABI MERAH (100GR)</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>🥓</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="n">
-        <v>158</v>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>PANGSIT GORENG</t>
-        </is>
-      </c>
-      <c r="E159" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t>PANGSIT GORENG (ISI 3)</t>
-        </is>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>🥟</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="n">
-        <v>159</v>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>BASO BABI GORENG</t>
-        </is>
-      </c>
-      <c r="E160" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F160" t="inlineStr">
-        <is>
-          <t>BASO BABI GORENG (2PCS)</t>
-        </is>
-      </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>🥟</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="n">
-        <v>160</v>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>BASO AYAM GORENG</t>
-        </is>
-      </c>
-      <c r="E161" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t>BASO AYAM GORENG (2PCS)</t>
-        </is>
-      </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>🥟</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="n">
-        <v>161</v>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>TELUR KECAP</t>
-        </is>
-      </c>
-      <c r="E162" t="n">
-        <v>3000</v>
-      </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>🥚</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="n">
-        <v>162</v>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>KERUPUK UDANG TOPING</t>
-        </is>
-      </c>
-      <c r="E163" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>KERUPUK UDANG</t>
-        </is>
-      </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>🍘</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="n">
-        <v>163</v>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>KERUPUK PUTIH TOPING</t>
-        </is>
-      </c>
-      <c r="E164" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t>KERUPUK PUTIH</t>
-        </is>
-      </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>🍘</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="n">
-        <v>164</v>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>TOPING TAMBAHAN</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>EMPING TOPING</t>
-        </is>
-      </c>
-      <c r="E165" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F165" t="inlineStr">
-        <is>
-          <t>EMPING</t>
-        </is>
-      </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>🍘</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="n">
-        <v>165</v>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>MINUMAN</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>BADAK</t>
-        </is>
-      </c>
-      <c r="E166" t="n">
-        <v>11000</v>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>🥤</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="n">
-        <v>166</v>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>MADAM LILY</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>MINUMAN</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>SONKIT</t>
-        </is>
-      </c>
-      <c r="E167" t="n">
-        <v>6000</v>
-      </c>
-      <c r="H167" t="inlineStr">
-        <is>
-          <t>🥤</t>
         </is>
       </c>
     </row>

</xml_diff>